<commit_message>
data(Gerencia): actualizar datos.xlsx y TALENTO HUMANO.xlsx (oficial)
</commit_message>
<xml_diff>
--- a/oficial/Gerencia/TALENTO HUMANO.xlsx
+++ b/oficial/Gerencia/TALENTO HUMANO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/FLUJO APP/APP_OPAUSTRO_OFICIAL/Gerencia/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ade4bf4107253254/OPAUSTRO DASHBOARD/TI OPAUSTRO/APP OPAUSTRO/APP OPAUSTRO/Gerencia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10ADF415-E820-4524-B9EB-F308C9A303B0}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{13C18F3D-9789-42FE-A96C-D3EBD5B9B8D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{996977CD-B87C-4485-A8E4-AA98CA6C457C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TALENTO ACTUAL" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="77">
   <si>
     <t>TALENTO HUMANO - SITUACION ACTUAL POR DEPARTAMENTO</t>
   </si>
@@ -242,6 +242,30 @@
   </si>
   <si>
     <t>Conducto inadecuada (Agresion)</t>
+  </si>
+  <si>
+    <t>JULIO</t>
+  </si>
+  <si>
+    <t>Rivera Ramos Jose</t>
+  </si>
+  <si>
+    <t>Feijoo Bayas Daniel Antonio</t>
+  </si>
+  <si>
+    <t>Soto Altamirano Jonathan</t>
+  </si>
+  <si>
+    <t>Contento Lagua Roberto</t>
+  </si>
+  <si>
+    <t>No asiste ala reunion vespertina</t>
+  </si>
+  <si>
+    <t>Se evidenció permanencia en su domicilio durante horas laborables y falta de visita a clientes.</t>
+  </si>
+  <si>
+    <t>Adulteracion de recibo de cobro</t>
   </si>
 </sst>
 </file>
@@ -814,13 +838,13 @@
         <v>14</v>
       </c>
       <c r="B4" s="16">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="C4" s="4">
         <v>79</v>
       </c>
       <c r="D4" s="4">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E4" s="4">
         <v>0</v>
@@ -833,15 +857,15 @@
       </c>
       <c r="H4" s="5">
         <f>C4-D4</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I4" s="6">
         <f>IF(C4=0,0,D4/C4)</f>
-        <v>0.97468354430379744</v>
+        <v>0.94936708860759489</v>
       </c>
       <c r="J4" s="6">
         <f>IF(D4=0,0,(F4+G4)/D4)</f>
-        <v>2.5974025974025976E-2</v>
+        <v>2.6666666666666668E-2</v>
       </c>
       <c r="K4" s="6">
         <f>4%</f>
@@ -857,7 +881,7 @@
         <v>15</v>
       </c>
       <c r="B5" s="16">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="C5" s="4">
         <v>22</v>
@@ -900,7 +924,7 @@
         <v>16</v>
       </c>
       <c r="B6" s="16">
-        <v>46203</v>
+        <v>46234</v>
       </c>
       <c r="C6" s="4">
         <v>29</v>
@@ -949,7 +973,7 @@
       </c>
       <c r="D7" s="9">
         <f t="shared" si="0"/>
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E7" s="9">
         <f t="shared" si="0"/>
@@ -965,15 +989,15 @@
       </c>
       <c r="H7" s="9">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I7" s="10">
         <f>IF(C7=0,0,D7/C7)</f>
-        <v>0.98461538461538467</v>
+        <v>0.96923076923076923</v>
       </c>
       <c r="J7" s="10">
         <f>IF(D7=0,0,(F7+G7)/D7)</f>
-        <v>2.34375E-2</v>
+        <v>2.3809523809523808E-2</v>
       </c>
       <c r="K7" s="10">
         <f>4%</f>
@@ -996,7 +1020,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1758,6 +1782,120 @@
         <v>6.8965517241379309E-2</v>
       </c>
     </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" s="11">
+        <v>75</v>
+      </c>
+      <c r="E22" s="11">
+        <v>2</v>
+      </c>
+      <c r="F22" s="11">
+        <v>4</v>
+      </c>
+      <c r="G22" s="11">
+        <v>3</v>
+      </c>
+      <c r="H22" s="11">
+        <v>3</v>
+      </c>
+      <c r="I22" s="13">
+        <f t="shared" ref="I22:I24" si="6">IF(D22=0,0,(E22+F22)/D22)</f>
+        <v>0.08</v>
+      </c>
+      <c r="J22" s="13">
+        <f t="shared" ref="J22:J24" si="7">IF(D22=0,0,E22/D22)</f>
+        <v>2.6666666666666668E-2</v>
+      </c>
+      <c r="K22" s="13">
+        <f t="shared" ref="K22:K24" si="8">IF(D22=0,0,F22/D22)</f>
+        <v>5.3333333333333337E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="D23" s="11">
+        <v>22</v>
+      </c>
+      <c r="E23" s="11">
+        <v>0</v>
+      </c>
+      <c r="F23" s="11">
+        <v>0</v>
+      </c>
+      <c r="G23" s="11">
+        <v>0</v>
+      </c>
+      <c r="H23" s="11">
+        <v>0</v>
+      </c>
+      <c r="I23" s="13">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="J23" s="13">
+        <f t="shared" si="7"/>
+        <v>0</v>
+      </c>
+      <c r="K23" s="13">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="11">
+        <v>2026</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D24" s="11">
+        <v>29</v>
+      </c>
+      <c r="E24" s="11">
+        <v>1</v>
+      </c>
+      <c r="F24" s="11">
+        <v>0</v>
+      </c>
+      <c r="G24" s="11">
+        <v>1</v>
+      </c>
+      <c r="H24" s="11">
+        <v>0</v>
+      </c>
+      <c r="I24" s="13">
+        <f t="shared" si="6"/>
+        <v>3.4482758620689655E-2</v>
+      </c>
+      <c r="J24" s="13">
+        <f t="shared" si="7"/>
+        <v>3.4482758620689655E-2</v>
+      </c>
+      <c r="K24" s="13">
+        <f t="shared" si="8"/>
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
@@ -1770,7 +1908,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2115,6 +2253,180 @@
       </c>
       <c r="J12" s="3"/>
     </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" s="16">
+        <v>46218</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H14" s="16">
+        <v>46218</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="H15" s="16">
+        <v>46211</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H16" s="16">
+        <v>46225</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H17" s="16">
+        <v>46225</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>2026</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="H18" s="16">
+        <v>46225</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>